<commit_message>
Rename "total mortality" -> "relative mortality" in all figure labels, tables, draft text, source data and HTML; figures/tables regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flux/paper_code_data/source_data/Fig2_net_mortality_shap_per_site.xlsx
+++ b/data/flux/paper_code_data/source_data/Fig2_net_mortality_shap_per_site.xlsx
@@ -23,7 +23,7 @@
     <t>Fig. 2: net signed SHAP of the mortality block per site (C+T+M, AutoGluon, 24 months).</t>
   </si>
   <si>
-    <t>Below zero = mortality lowers the predicted property. Sites ordered by total_mortality_site_max_pct.</t>
+    <t>Below zero = mortality lowers the predicted property. Sites ordered by relative_mortality_site_max_pct.</t>
   </si>
   <si>
     <t>SITE_ID</t>
@@ -38,7 +38,7 @@
     <t>net_mortality_shap</t>
   </si>
   <si>
-    <t>total_mortality_site_max_pct</t>
+    <t>relative_mortality_site_max_pct</t>
   </si>
   <si>
     <t>mortality_class</t>

</xml_diff>